<commit_message>
Use unique group numbers across both Cores
</commit_message>
<xml_diff>
--- a/data/E-Vocab-Band-II-Core-I.xlsx
+++ b/data/E-Vocab-Band-II-Core-I.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core I Data" sheetId="1" r:id="Rf7c309c0eb0541bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method &amp; Sources" sheetId="2" r:id="Red4983e956c246e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core I Data" sheetId="1" r:id="R4a4f6a9650344849"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method &amp; Sources" sheetId="2" r:id="R445c2fd09bca40f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -50319,7 +50319,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R757e47dd20e24e1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra24ad868d8e7482a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -50484,10 +50484,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="43" t="str">
-        <x:v>Number of groups</x:v>
-      </x:c>
-      <x:c r="B13" s="44" t="n">
-        <x:v>20</x:v>
+        <x:v>Group number range</x:v>
+      </x:c>
+      <x:c r="B13" s="44" t="str">
+        <x:v>1–20</x:v>
       </x:c>
       <x:c r="C13" s="40"/>
       <x:c r="D13" s="40"/>
@@ -50600,7 +50600,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="38" t="str">
-        <x:v>7. Records were randomly shuffled within Core I, then assigned sequentially to 20 near-equal groups. Shuffle seed: 144dc3776adf83833cb36b58d887de5deb59ebeab2a8cf95fffbdb609b1f2518</x:v>
+        <x:v>7. Records were randomly shuffled within Core I, then assigned sequentially to near-equal groups 1–20. Shuffle seed: 144dc3776adf83833cb36b58d887de5deb59ebeab2a8cf95fffbdb609b1f2518</x:v>
       </x:c>
       <x:c r="B24" s="38"/>
       <x:c r="C24" s="38"/>

</xml_diff>